<commit_message>
Page « Et si on enlevait tous les passages à niveau? » (sensibilité 241 km/h)
Demande client : une page unique pour juger si la dénivellation complète vaut
l'investissement. Bande 241 (150 mi/h, plafond prouvé du NEC sous ACSES,
fra2010ptc/fra2000acela) ajoutée au moteur 21 (même rame pendulaire 12 W/kg,
lecture conservatrice) ; les trois CSV de scénarios portent la bande.

Verdict de la page : lever le mur des 924 passages n'achète que 2 à 12 min par
trajet (16 min Québec-Toronto de bout en bout) parce qu'au-dessus de 201 ce
sont les courbes qui retiennent le train. Comme levier de temps, ça ne se
justifie pas ; les minutes au-delà du scénario 3 exigent de toucher au tracé,
c'est-à-dire le projet d'ALTO. Section d'une page (p. 17), surtitre « La
contre-hypothèse », PDF 22 pages.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/livrables/decomposition_gains.xlsx
+++ b/livrables/decomposition_gains.xlsx
@@ -476,7 +476,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>392.8</v>
+        <v>370</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -496,10 +496,10 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>15.7</v>
+        <v>30</v>
       </c>
       <c r="D3" t="n">
-        <v>11.4</v>
+        <v>18.7</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -519,10 +519,10 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>35.4</v>
+        <v>38.2</v>
       </c>
       <c r="D4" t="n">
-        <v>25.7</v>
+        <v>23.8</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -542,10 +542,10 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>42.4</v>
+        <v>42.6</v>
       </c>
       <c r="D5" t="n">
-        <v>30.8</v>
+        <v>26.5</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -565,10 +565,10 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>14.2</v>
+        <v>19.7</v>
       </c>
       <c r="D6" t="n">
-        <v>10.3</v>
+        <v>12.3</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -591,7 +591,7 @@
         <v>22.1</v>
       </c>
       <c r="D7" t="n">
-        <v>16.1</v>
+        <v>13.8</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -614,7 +614,7 @@
         <v>7.9</v>
       </c>
       <c r="D8" t="n">
-        <v>5.7</v>
+        <v>4.9</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -654,7 +654,7 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>137.7</v>
+        <v>160.5</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -674,7 +674,7 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>4.8</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -694,7 +694,7 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>125.7</v>
+        <v>116.1</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -714,10 +714,10 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>3.9</v>
+        <v>7</v>
       </c>
       <c r="D13" t="n">
-        <v>5</v>
+        <v>8.1</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -737,10 +737,10 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>15.5</v>
+        <v>16.5</v>
       </c>
       <c r="D14" t="n">
-        <v>20.2</v>
+        <v>19.1</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -763,7 +763,7 @@
         <v>19.6</v>
       </c>
       <c r="D15" t="n">
-        <v>25.5</v>
+        <v>22.6</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -783,10 +783,10 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>14.2</v>
+        <v>19.7</v>
       </c>
       <c r="D16" t="n">
-        <v>18.5</v>
+        <v>22.8</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -809,7 +809,7 @@
         <v>22.1</v>
       </c>
       <c r="D17" t="n">
-        <v>28.8</v>
+        <v>25.6</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -832,7 +832,7 @@
         <v>1.5</v>
       </c>
       <c r="D18" t="n">
-        <v>2</v>
+        <v>1.8</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -872,7 +872,7 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>76.8</v>
+        <v>86.40000000000001</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -892,7 +892,7 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>1.6</v>
+        <v>3.4</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -912,7 +912,7 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>88.59999999999999</v>
+        <v>82.59999999999999</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
@@ -932,10 +932,10 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>1.2</v>
+        <v>2.4</v>
       </c>
       <c r="D23" t="n">
-        <v>3.7</v>
+        <v>6</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -955,10 +955,10 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>9.4</v>
+        <v>9.9</v>
       </c>
       <c r="D24" t="n">
-        <v>28.2</v>
+        <v>25.3</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -978,10 +978,10 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>15.6</v>
+        <v>15.7</v>
       </c>
       <c r="D25" t="n">
-        <v>46.7</v>
+        <v>39.9</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
@@ -1001,10 +1001,10 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>7.1</v>
+        <v>11.3</v>
       </c>
       <c r="D26" t="n">
-        <v>21.4</v>
+        <v>28.8</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
@@ -1090,7 +1090,7 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>33.4</v>
+        <v>39.4</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -1110,7 +1110,7 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>0.6</v>
+        <v>1</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>

</xml_diff>